<commit_message>
Fill sole-proprietor identity into contract and invoice drafts
Store unvan, Van tax office VKN and NACE codes (excluding programming)
for fatura/sözleşme use; omit TCKN from the repo.

Co-authored-by: barsokrr <barsokrr@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/metraj/Fatura_Kesim_Formu_Kalip_Hakedis.xlsx
+++ b/metraj/Fatura_Kesim_Formu_Kalip_Hakedis.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>…………………… (Şahıs Şirketi)</t>
+          <t>ABDURRAHMAN BARIŞ ÖKER (şahıs / gerçek kişi)</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>…………………… / ………………</t>
+          <t>Van Vergi Dairesi Müd. / 6530560679</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>43.99.05</t>
+          <t>43.99.05 (ayrıca 71.11.01 kayıtlı)</t>
         </is>
       </c>
     </row>
@@ -1153,9 +1153,9 @@
   </sheetData>
   <mergeCells count="23">
     <mergeCell ref="A34:H36"/>
+    <mergeCell ref="B40:H40"/>
+    <mergeCell ref="B7:C7"/>
     <mergeCell ref="F5:H5"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B40:H40"/>
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B45:H45"/>

</xml_diff>